<commit_message>
Add a bar chart of the schedule to the Gantt workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S6mvbXzTvRoGpVPUkaDb65
</commit_message>
<xml_diff>
--- a/report/Gantt_Chart.xlsx
+++ b/report/Gantt_Chart.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gantt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -186,6 +187,338 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Project schedule</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Chart data'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Chart data'!$A$2:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Chart data'!$B$2:$B$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Chart data'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="4A78B5"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4C9A6A"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4C9A6A"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4C9A6A"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4C9A6A"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="5"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="7"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="8"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="9"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="10"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="11"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="4A78B5"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="12"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="C0392B"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="13"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="C0392B"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="14"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="C0392B"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="15"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="C0392B"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'Chart data'!$A$2:$A$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Chart data'!$C$2:$C$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="40"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="26"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Week (1-13 Trimester 1, 14 break, 15-26 Trimester 2)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <majorUnit val="1"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10800000" cy="4680000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1570,7 +1903,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Final technical report</t>
+          <t>Final technical report due</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1662,4 +1995,339 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Colour</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Literature review and project proposal</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Requirements and review of SSMC records</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data model design</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Application build (HV overview, SLD generation)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Breaker status, maintenance records, history</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Named user logins and hosted demonstration</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Data entry of LVSB room records</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>On-site verification of 10 entries</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Poster preparation</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Timed lookup evaluation</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>18</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Refinement from evaluation results</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>19</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Final technical report</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C13" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Project proposal (25 Oct)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Poster presentation</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>17</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Final demonstration</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Final technical report due</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Week numbers: 1-13 = Trimester 1 W1-W13, 14 = term break, 15-26 = Trimester 2 W1-W12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>